<commit_message>
auditor: RGF semestral e quadrimestral lado a lado (quadros 6 e 7)
- Tela: volta os slots RGF 1o/2o Semestre ao lado dos 3 quadrimestres.
- Status: Q6/Q7 ficam completos com o modelo quadrimestral ou o semestral
  (docs_alternativos), no site e na aba Status do Excel.
- Q6/Q7 (Excel e RIT): cabecalhos seguem o periodo do RGF enviado
  (2o Quadrimestre / 1o Semestre; colunas do Q7 por quadrimestre ou semestre).
  Planilhas antigas com chaves semestrais continuam gerando o RIT.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend-auditor/templates/quadro_07.xlsx
+++ b/backend-auditor/templates/quadro_07.xlsx
@@ -681,17 +681,17 @@
       <c r="B5" s="17" t="n"/>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Até o 1º Quadrimestre</t>
+          <t>{rotulos.col_1}</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Até o 2º Quadrimestre</t>
+          <t>{rotulos.col_2}</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Até o 3º Quadrimestre</t>
+          <t>{rotulos.col_3}</t>
         </is>
       </c>
     </row>

</xml_diff>